<commit_message>
updating repository to local
</commit_message>
<xml_diff>
--- a/public/files/Data_By_Towns_Index/Burlington/Beverly City.xlsx
+++ b/public/files/Data_By_Towns_Index/Burlington/Beverly City.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,168 +425,125 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Unnamed: 0</t>
+          <t>Owner Name</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Owner Name</t>
+          <t>Property Location</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Property Location</t>
+          <t>Municipality</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Municipality</t>
+          <t>County</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Search</t>
+          <t>State</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>Longitude</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>Latitude</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Longitude</t>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>PID</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
-        <v>0</v>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>SHAH, JUNAID</t>
+        </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>PATEL, GAURAV AND NIKITABEN</t>
+          <t>618 WARREN ST</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>222 COOPER ST</t>
+          <t>Beverly City</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Beverly City</t>
+          <t>Burlington</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Patel</t>
+          <t>NJ</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>40.0659381</v>
+        <v>-74.92327019999999</v>
       </c>
       <c r="G2" t="n">
-        <v>-74.91946039999999</v>
+        <v>40.06356359999999</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>ChIJJxb9LopMwYkRWgjcW_yTOBs</t>
+        </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
-        <v>1</v>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>SHAH, MUBINA &amp; KHAN, MOHAMMED N</t>
+        </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>SHAH, JUNA D &amp; PIA, SEFAT</t>
+          <t>226-228 LAUREL ST</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>28 PINE STREET</t>
+          <t>Beverly City</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Beverly City</t>
+          <t>Burlington</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Shah</t>
+          <t>NJ</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>40.0627701</v>
+        <v>-74.920395</v>
       </c>
       <c r="G3" t="n">
-        <v>-74.9123183</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>2</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>SHAH, JUNAID</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>618 WARREN ST</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Beverly City</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Shah</t>
-        </is>
-      </c>
-      <c r="F4" t="n">
-        <v>40.06356359999999</v>
-      </c>
-      <c r="G4" t="n">
-        <v>-74.92327019999999</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>3</v>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>SHAH, MUBINA &amp; KHAN, MOHAMMED N</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>226-228 LAUREL ST</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Beverly City</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Shah</t>
-        </is>
-      </c>
-      <c r="F5" t="n">
         <v>40.065744</v>
       </c>
-      <c r="G5" t="n">
-        <v>-74.920395</v>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>ChIJ4wUcL2BMwYkRi104CXUPMbI</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>